<commit_message>
change to DB and add auto refresh token func
</commit_message>
<xml_diff>
--- a/TESTt.xlsx
+++ b/TESTt.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\งาน\ฝึกงาน BOTNOI\calendarAPI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7EF84A1-D03F-4FC5-9340-2F3A01E0F5A7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{473E9766-91D8-4F8B-A61E-081D82994C54}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="M" sheetId="1" r:id="rId1"/>
@@ -29023,9 +29023,9 @@
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1" xr:uid="{31A93216-10CA-4192-A918-EB023B2FB873}"/>
-    <hyperlink ref="B5" r:id="rId2" xr:uid="{FC5FD774-7CC6-4EDC-BD22-7522D421BB78}"/>
-    <hyperlink ref="B7" r:id="rId3" xr:uid="{23DAC81B-1342-4CEE-89F1-6BF0B5FB02B0}"/>
+    <hyperlink ref="B5" r:id="rId1" xr:uid="{FC5FD774-7CC6-4EDC-BD22-7522D421BB78}"/>
+    <hyperlink ref="B7" r:id="rId2" xr:uid="{23DAC81B-1342-4CEE-89F1-6BF0B5FB02B0}"/>
+    <hyperlink ref="B6" r:id="rId3" xr:uid="{31A93216-10CA-4192-A918-EB023B2FB873}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>